<commit_message>
feat(forms): add plain-language Word returns and visible team prefills
</commit_message>
<xml_diff>
--- a/docs/forms/OHCS-Q3-2026-Team-Maintenance-Form.xlsx
+++ b/docs/forms/OHCS-Q3-2026-Team-Maintenance-Form.xlsx
@@ -3,6 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12000" windowHeight="9000" firstSheet="0" activeTab="1"/>
+  </bookViews>
   <sheets>
     <sheet sheetId="1" name="Instructions" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Team" state="visible" r:id="rId5"/>
@@ -22,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="84">
   <si>
     <t>OHCS TEAM MAINTENANCE FORM</t>
   </si>
@@ -30,6 +33,24 @@
     <t>How to complete</t>
   </si>
   <si>
+    <t>YOUR TEAM</t>
+  </si>
+  <si>
+    <t>Enter your team name on the Team tab</t>
+  </si>
+  <si>
+    <t>PARTICIPATING OFFICERS</t>
+  </si>
+  <si>
+    <t>Enter participating officers on the Team tab</t>
+  </si>
+  <si>
+    <t>REPORTING PERIOD</t>
+  </si>
+  <si>
+    <t>Q3 2026 — actual visit dates are recorded separately</t>
+  </si>
+  <si>
     <t>1. Team</t>
   </si>
   <si>
@@ -105,7 +126,7 @@
     <t>Workbook ID</t>
   </si>
   <si>
-    <t>c5b325b6-6f84-4c8c-8485-7c8ce4c17599</t>
+    <t>90de6f18-5f3e-45f3-ae6f-5f808e967401</t>
   </si>
   <si>
     <t>Reporting year</t>
@@ -697,7 +718,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" style="1" customWidth="1"/>
@@ -790,6 +811,30 @@
       </c>
       <c r="B11" s="3" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" ht="50" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" ht="50" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -813,82 +858,82 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -899,6 +944,10 @@
   <autoFilter ref="A1:B11"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddHeader>&amp;L
+&amp;RQ3 2026</oddHeader>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -919,22 +968,22 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -1355,6 +1404,10 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddHeader>&amp;L
+&amp;RQ3 2026</oddHeader>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1381,46 +1434,46 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" ht="48" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -3047,6 +3100,10 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="2" fitToHeight="0"/>
+  <headerFooter>
+    <oddHeader>&amp;L
+&amp;RQ3 2026</oddHeader>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -3064,98 +3121,98 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>